<commit_message>
Feb 24th FINAL CODE
</commit_message>
<xml_diff>
--- a/Code/1. Exploratory Data Analysis/near_constant_columns_90pct.xlsx
+++ b/Code/1. Exploratory Data Analysis/near_constant_columns_90pct.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E110"/>
+  <dimension ref="A1:E109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3 (60950-21)</t>
+          <t>2 (EN 60950/EN 60065)</t>
         </is>
       </c>
       <c r="B2" t="b">
@@ -465,7 +465,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>5 (60950-23)</t>
+          <t>3 (60950-21)</t>
         </is>
       </c>
       <c r="B3" t="b">
@@ -484,7 +484,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2 (EN 60950/EN 60065)</t>
+          <t>BSMI</t>
         </is>
       </c>
       <c r="B4" t="b">
@@ -503,7 +503,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BSMI</t>
+          <t>5 (60950-23)</t>
         </is>
       </c>
       <c r="B5" t="b">
@@ -522,7 +522,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NOM</t>
+          <t>PSE</t>
         </is>
       </c>
       <c r="B6" t="b">
@@ -560,7 +560,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PSE</t>
+          <t>NOM</t>
         </is>
       </c>
       <c r="B8" t="b">
@@ -579,17 +579,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>type_of_investigation_Missing</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+          <t>CCC</t>
+        </is>
+      </c>
+      <c r="B9" t="b">
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>1823</v>
+        <v>1822</v>
       </c>
       <c r="D9" t="n">
-        <v>99.95</v>
+        <v>99.89</v>
       </c>
       <c r="E9" t="n">
         <v>2</v>
@@ -598,17 +598,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>Test- Bridging Resistor Test</t>
         </is>
       </c>
       <c r="B10" t="b">
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>1822</v>
+        <v>1821</v>
       </c>
       <c r="D10" t="n">
-        <v>99.89</v>
+        <v>99.84</v>
       </c>
       <c r="E10" t="n">
         <v>2</v>
@@ -617,7 +617,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Test- Bridging Resistor Test</t>
+          <t>multilayer_boards</t>
         </is>
       </c>
       <c r="B11" t="b">
@@ -636,7 +636,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>102 (LFC)</t>
+          <t>thin_material_test</t>
         </is>
       </c>
       <c r="B12" t="b">
@@ -655,7 +655,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>thin_material_test</t>
+          <t>102 (LFC)</t>
         </is>
       </c>
       <c r="B13" t="b">
@@ -674,17 +674,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>multilayer_boards</t>
-        </is>
-      </c>
-      <c r="B14" t="b">
+          <t>total_schemmes</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>1821</v>
+        <v>1820</v>
       </c>
       <c r="D14" t="n">
-        <v>99.84</v>
+        <v>99.78</v>
       </c>
       <c r="E14" t="n">
         <v>2</v>
@@ -712,17 +712,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>total_schemmes</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+          <t>dust_test</t>
+        </is>
+      </c>
+      <c r="B16" t="b">
         <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="D16" t="n">
-        <v>99.78</v>
+        <v>99.73</v>
       </c>
       <c r="E16" t="n">
         <v>2</v>
@@ -731,17 +731,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>dust_test</t>
+          <t>unknown_PWR_supply</t>
         </is>
       </c>
       <c r="B17" t="b">
         <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>1819</v>
+        <v>1817</v>
       </c>
       <c r="D17" t="n">
-        <v>99.73</v>
+        <v>99.62</v>
       </c>
       <c r="E17" t="n">
         <v>2</v>
@@ -750,7 +750,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>unknown_PWR_supply</t>
+          <t>uncertified_pwr_supply</t>
         </is>
       </c>
       <c r="B18" t="b">
@@ -769,17 +769,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>uncertified_pwr_supply</t>
+          <t>energy_hazard_test</t>
         </is>
       </c>
       <c r="B19" t="b">
         <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>1817</v>
+        <v>1816</v>
       </c>
       <c r="D19" t="n">
-        <v>99.62</v>
+        <v>99.56</v>
       </c>
       <c r="E19" t="n">
         <v>2</v>
@@ -807,17 +807,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>energy_hazard_test</t>
+          <t>Test- Secondary Working Voltage</t>
         </is>
       </c>
       <c r="B21" t="b">
         <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>1816</v>
+        <v>1815</v>
       </c>
       <c r="D21" t="n">
-        <v>99.56</v>
+        <v>99.51000000000001</v>
       </c>
       <c r="E21" t="n">
         <v>2</v>
@@ -826,7 +826,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>moment_test</t>
+          <t>alter_strain_relief</t>
         </is>
       </c>
       <c r="B22" t="b">
@@ -845,10 +845,10 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CCN_Top10_NWIN</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
+          <t>alter_relay</t>
+        </is>
+      </c>
+      <c r="B23" t="b">
         <v>0</v>
       </c>
       <c r="C23" t="n">
@@ -864,10 +864,10 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>alter_strain_relief</t>
-        </is>
-      </c>
-      <c r="B24" t="b">
+          <t>CCN_Top10_NWIN</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
         <v>0</v>
       </c>
       <c r="C24" t="n">
@@ -902,7 +902,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>alter_relay</t>
+          <t>moment_test</t>
         </is>
       </c>
       <c r="B26" t="b">
@@ -921,17 +921,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Test- Secondary Working Voltage</t>
+          <t>outdoor_use</t>
         </is>
       </c>
       <c r="B27" t="b">
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>1815</v>
+        <v>1814</v>
       </c>
       <c r="D27" t="n">
-        <v>99.51000000000001</v>
+        <v>99.45</v>
       </c>
       <c r="E27" t="n">
         <v>2</v>
@@ -959,17 +959,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>outdoor_use</t>
+          <t>Test- Tensile Strength</t>
         </is>
       </c>
       <c r="B29" t="b">
         <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>1814</v>
+        <v>1813</v>
       </c>
       <c r="D29" t="n">
-        <v>99.45</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E29" t="n">
         <v>2</v>
@@ -978,7 +978,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Test- Tensile Strength</t>
+          <t>PoE_source</t>
         </is>
       </c>
       <c r="B30" t="b">
@@ -1016,17 +1016,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>PoE_source</t>
+          <t>7 (950 TO 368)</t>
         </is>
       </c>
       <c r="B32" t="b">
         <v>0</v>
       </c>
       <c r="C32" t="n">
-        <v>1813</v>
+        <v>1812</v>
       </c>
       <c r="D32" t="n">
-        <v>99.40000000000001</v>
+        <v>99.34</v>
       </c>
       <c r="E32" t="n">
         <v>2</v>
@@ -1035,17 +1035,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7 (950 TO 368)</t>
+          <t>alter_movs</t>
         </is>
       </c>
       <c r="B33" t="b">
         <v>0</v>
       </c>
       <c r="C33" t="n">
-        <v>1812</v>
+        <v>1811</v>
       </c>
       <c r="D33" t="n">
-        <v>99.34</v>
+        <v>99.29000000000001</v>
       </c>
       <c r="E33" t="n">
         <v>2</v>
@@ -1054,7 +1054,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>alter_movs</t>
+          <t>alter_app_inlet</t>
         </is>
       </c>
       <c r="B34" t="b">
@@ -1073,10 +1073,10 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>alter_app_inlet</t>
-        </is>
-      </c>
-      <c r="B35" t="b">
+          <t>type_of_investigation_5 - Administrative CB review</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
         <v>0</v>
       </c>
       <c r="C35" t="n">
@@ -1092,17 +1092,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>type_of_investigation_5 - Administrative CB review</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
+          <t>alter_resistor</t>
+        </is>
+      </c>
+      <c r="B36" t="b">
         <v>0</v>
       </c>
       <c r="C36" t="n">
-        <v>1811</v>
+        <v>1810</v>
       </c>
       <c r="D36" t="n">
-        <v>99.29000000000001</v>
+        <v>99.23</v>
       </c>
       <c r="E36" t="n">
         <v>2</v>
@@ -1111,7 +1111,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>alter_resistor</t>
+          <t>all_mount_test</t>
         </is>
       </c>
       <c r="B37" t="b">
@@ -1130,17 +1130,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>all_mount_test</t>
+          <t>alter_LPS</t>
         </is>
       </c>
       <c r="B38" t="b">
         <v>0</v>
       </c>
       <c r="C38" t="n">
-        <v>1810</v>
+        <v>1809</v>
       </c>
       <c r="D38" t="n">
-        <v>99.23</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="E38" t="n">
         <v>2</v>
@@ -1149,10 +1149,10 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>alter_LPS</t>
-        </is>
-      </c>
-      <c r="B39" t="b">
+          <t>CCN_Top10_QQGQ2</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
         <v>0</v>
       </c>
       <c r="C39" t="n">
@@ -1168,10 +1168,10 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CCN_Top10_QQGQ2</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
+          <t>alter_display</t>
+        </is>
+      </c>
+      <c r="B40" t="b">
         <v>0</v>
       </c>
       <c r="C40" t="n">
@@ -1206,17 +1206,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>alter_display</t>
+          <t>alter_light</t>
         </is>
       </c>
       <c r="B42" t="b">
         <v>0</v>
       </c>
       <c r="C42" t="n">
-        <v>1809</v>
+        <v>1808</v>
       </c>
       <c r="D42" t="n">
-        <v>99.18000000000001</v>
+        <v>99.12</v>
       </c>
       <c r="E42" t="n">
         <v>2</v>
@@ -1244,17 +1244,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>alter_light</t>
+          <t>stability_test</t>
         </is>
       </c>
       <c r="B44" t="b">
         <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>1808</v>
+        <v>1807</v>
       </c>
       <c r="D44" t="n">
-        <v>99.12</v>
+        <v>99.06999999999999</v>
       </c>
       <c r="E44" t="n">
         <v>2</v>
@@ -1320,17 +1320,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>stability_test</t>
+          <t>alter_optical_isolator</t>
         </is>
       </c>
       <c r="B48" t="b">
         <v>0</v>
       </c>
       <c r="C48" t="n">
-        <v>1807</v>
+        <v>1806</v>
       </c>
       <c r="D48" t="n">
-        <v>99.06999999999999</v>
+        <v>99.01000000000001</v>
       </c>
       <c r="E48" t="n">
         <v>2</v>
@@ -1339,17 +1339,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>alter_optical_isolator</t>
+          <t>PoE_load</t>
         </is>
       </c>
       <c r="B49" t="b">
         <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>1806</v>
+        <v>1805</v>
       </c>
       <c r="D49" t="n">
-        <v>99.01000000000001</v>
+        <v>98.95999999999999</v>
       </c>
       <c r="E49" t="n">
         <v>2</v>
@@ -1358,17 +1358,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PoE_load</t>
-        </is>
-      </c>
-      <c r="B50" t="b">
+          <t>CCN_Top10_AAAL</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
         <v>0</v>
       </c>
       <c r="C50" t="n">
-        <v>1805</v>
+        <v>1804</v>
       </c>
       <c r="D50" t="n">
-        <v>98.95999999999999</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="E50" t="n">
         <v>2</v>
@@ -1396,17 +1396,18 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CCN_Top10_AAAL</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
+          <t xml:space="preserve">
+33 (Rename)</t>
+        </is>
+      </c>
+      <c r="B52" t="b">
         <v>0</v>
       </c>
       <c r="C52" t="n">
-        <v>1804</v>
+        <v>1802</v>
       </c>
       <c r="D52" t="n">
-        <v>98.90000000000001</v>
+        <v>98.79000000000001</v>
       </c>
       <c r="E52" t="n">
         <v>2</v>
@@ -1415,18 +1416,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">
-33 (Rename)</t>
+          <t>alter_fuse</t>
         </is>
       </c>
       <c r="B53" t="b">
         <v>0</v>
       </c>
       <c r="C53" t="n">
-        <v>1802</v>
+        <v>1800</v>
       </c>
       <c r="D53" t="n">
-        <v>98.79000000000001</v>
+        <v>98.68000000000001</v>
       </c>
       <c r="E53" t="n">
         <v>2</v>
@@ -1435,17 +1435,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>alter_fuse</t>
+          <t>alter_complex</t>
         </is>
       </c>
       <c r="B54" t="b">
         <v>0</v>
       </c>
       <c r="C54" t="n">
-        <v>1800</v>
+        <v>1799</v>
       </c>
       <c r="D54" t="n">
-        <v>98.68000000000001</v>
+        <v>98.63</v>
       </c>
       <c r="E54" t="n">
         <v>2</v>
@@ -1454,17 +1454,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>alter_complex</t>
+          <t>family_grouping</t>
         </is>
       </c>
       <c r="B55" t="b">
         <v>0</v>
       </c>
       <c r="C55" t="n">
-        <v>1799</v>
+        <v>1797</v>
       </c>
       <c r="D55" t="n">
-        <v>98.63</v>
+        <v>98.52</v>
       </c>
       <c r="E55" t="n">
         <v>2</v>
@@ -1492,17 +1492,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>family_grouping</t>
+          <t>power_measurement_test</t>
         </is>
       </c>
       <c r="B57" t="b">
         <v>0</v>
       </c>
       <c r="C57" t="n">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="D57" t="n">
-        <v>98.52</v>
+        <v>98.45999999999999</v>
       </c>
       <c r="E57" t="n">
         <v>2</v>
@@ -1511,17 +1511,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>power_measurement_test</t>
+          <t>alter_connector</t>
         </is>
       </c>
       <c r="B58" t="b">
         <v>0</v>
       </c>
       <c r="C58" t="n">
-        <v>1796</v>
+        <v>1795</v>
       </c>
       <c r="D58" t="n">
-        <v>98.45999999999999</v>
+        <v>98.41</v>
       </c>
       <c r="E58" t="n">
         <v>2</v>
@@ -1549,17 +1549,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>alter_connector</t>
-        </is>
-      </c>
-      <c r="B60" t="b">
+          <t>CCN_Top10_AAAU</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
         <v>0</v>
       </c>
       <c r="C60" t="n">
-        <v>1795</v>
+        <v>1794</v>
       </c>
       <c r="D60" t="n">
-        <v>98.41</v>
+        <v>98.36</v>
       </c>
       <c r="E60" t="n">
         <v>2</v>
@@ -1568,17 +1568,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CCN_Top10_AAAU</t>
+          <t>CCN_Top10_AALL</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>0</v>
       </c>
       <c r="C61" t="n">
-        <v>1794</v>
+        <v>1790</v>
       </c>
       <c r="D61" t="n">
-        <v>98.36</v>
+        <v>98.14</v>
       </c>
       <c r="E61" t="n">
         <v>2</v>
@@ -1606,17 +1606,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CCN_Top10_AALL</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
+          <t>alter_transformer</t>
+        </is>
+      </c>
+      <c r="B63" t="b">
         <v>0</v>
       </c>
       <c r="C63" t="n">
-        <v>1790</v>
+        <v>1789</v>
       </c>
       <c r="D63" t="n">
-        <v>98.14</v>
+        <v>98.08</v>
       </c>
       <c r="E63" t="n">
         <v>2</v>
@@ -1625,17 +1625,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>alter_transformer</t>
+          <t>IT Informational Test Report</t>
         </is>
       </c>
       <c r="B64" t="b">
         <v>0</v>
       </c>
       <c r="C64" t="n">
-        <v>1789</v>
+        <v>1788</v>
       </c>
       <c r="D64" t="n">
-        <v>98.08</v>
+        <v>98.03</v>
       </c>
       <c r="E64" t="n">
         <v>2</v>
@@ -1644,17 +1644,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>IT Informational Test Report</t>
+          <t>loading_wall_test</t>
         </is>
       </c>
       <c r="B65" t="b">
         <v>0</v>
       </c>
       <c r="C65" t="n">
-        <v>1788</v>
+        <v>1787</v>
       </c>
       <c r="D65" t="n">
-        <v>98.03</v>
+        <v>97.97</v>
       </c>
       <c r="E65" t="n">
         <v>2</v>
@@ -1663,17 +1663,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>loading_wall_test</t>
+          <t>batt_drop_test</t>
         </is>
       </c>
       <c r="B66" t="b">
         <v>0</v>
       </c>
       <c r="C66" t="n">
-        <v>1787</v>
+        <v>1786</v>
       </c>
       <c r="D66" t="n">
-        <v>97.97</v>
+        <v>97.92</v>
       </c>
       <c r="E66" t="n">
         <v>2</v>
@@ -1701,17 +1701,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>batt_drop_test</t>
+          <t>XFR_abnormal_operation_test</t>
         </is>
       </c>
       <c r="B68" t="b">
         <v>0</v>
       </c>
       <c r="C68" t="n">
-        <v>1786</v>
+        <v>1783</v>
       </c>
       <c r="D68" t="n">
-        <v>97.92</v>
+        <v>97.75</v>
       </c>
       <c r="E68" t="n">
         <v>2</v>
@@ -1720,7 +1720,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>XFR_abnormal_operation_test</t>
+          <t>protective_bondingII_test</t>
         </is>
       </c>
       <c r="B69" t="b">
@@ -1739,17 +1739,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>protective_bondingII_test</t>
+          <t>max_output_test</t>
         </is>
       </c>
       <c r="B70" t="b">
         <v>0</v>
       </c>
       <c r="C70" t="n">
-        <v>1783</v>
+        <v>1782</v>
       </c>
       <c r="D70" t="n">
-        <v>97.75</v>
+        <v>97.7</v>
       </c>
       <c r="E70" t="n">
         <v>2</v>
@@ -1777,17 +1777,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>max_output_test</t>
+          <t>alter_capacitor</t>
         </is>
       </c>
       <c r="B72" t="b">
         <v>0</v>
       </c>
       <c r="C72" t="n">
-        <v>1782</v>
+        <v>1780</v>
       </c>
       <c r="D72" t="n">
-        <v>97.7</v>
+        <v>97.59</v>
       </c>
       <c r="E72" t="n">
         <v>2</v>
@@ -1796,17 +1796,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>alter_capacitor</t>
+          <t>enclosure_push_test</t>
         </is>
       </c>
       <c r="B73" t="b">
         <v>0</v>
       </c>
       <c r="C73" t="n">
-        <v>1780</v>
+        <v>1779</v>
       </c>
       <c r="D73" t="n">
-        <v>97.59</v>
+        <v>97.53</v>
       </c>
       <c r="E73" t="n">
         <v>2</v>
@@ -1834,17 +1834,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>enclosure_push_test</t>
+          <t>alter_current_ic</t>
         </is>
       </c>
       <c r="B75" t="b">
         <v>0</v>
       </c>
       <c r="C75" t="n">
-        <v>1779</v>
+        <v>1778</v>
       </c>
       <c r="D75" t="n">
-        <v>97.53</v>
+        <v>97.48</v>
       </c>
       <c r="E75" t="n">
         <v>2</v>
@@ -1853,17 +1853,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>alter_current_ic</t>
+          <t>30 (Talk to Derek)</t>
         </is>
       </c>
       <c r="B76" t="b">
         <v>0</v>
       </c>
       <c r="C76" t="n">
-        <v>1778</v>
+        <v>1774</v>
       </c>
       <c r="D76" t="n">
-        <v>97.48</v>
+        <v>97.26000000000001</v>
       </c>
       <c r="E76" t="n">
         <v>2</v>
@@ -1872,17 +1872,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>30 (Talk to Derek)</t>
+          <t>LCC_test</t>
         </is>
       </c>
       <c r="B77" t="b">
         <v>0</v>
       </c>
       <c r="C77" t="n">
-        <v>1774</v>
+        <v>1773</v>
       </c>
       <c r="D77" t="n">
-        <v>97.26000000000001</v>
+        <v>97.2</v>
       </c>
       <c r="E77" t="n">
         <v>2</v>
@@ -1891,17 +1891,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>LCC_test</t>
+          <t>CB_reissue</t>
         </is>
       </c>
       <c r="B78" t="b">
         <v>0</v>
       </c>
       <c r="C78" t="n">
-        <v>1773</v>
+        <v>1772</v>
       </c>
       <c r="D78" t="n">
-        <v>97.2</v>
+        <v>97.15000000000001</v>
       </c>
       <c r="E78" t="n">
         <v>2</v>
@@ -1910,7 +1910,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CB_reissue</t>
+          <t>XFR_strength_test</t>
         </is>
       </c>
       <c r="B79" t="b">
@@ -1929,17 +1929,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>XFR_strength_test</t>
+          <t>PS_shortcircuit_test</t>
         </is>
       </c>
       <c r="B80" t="b">
         <v>0</v>
       </c>
       <c r="C80" t="n">
-        <v>1772</v>
+        <v>1759</v>
       </c>
       <c r="D80" t="n">
-        <v>97.15000000000001</v>
+        <v>96.44</v>
       </c>
       <c r="E80" t="n">
         <v>2</v>
@@ -1948,17 +1948,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>PS_shortcircuit_test</t>
+          <t>34 (may be duplicate - check)</t>
         </is>
       </c>
       <c r="B81" t="b">
         <v>0</v>
       </c>
       <c r="C81" t="n">
-        <v>1759</v>
+        <v>1751</v>
       </c>
       <c r="D81" t="n">
-        <v>96.44</v>
+        <v>96</v>
       </c>
       <c r="E81" t="n">
         <v>2</v>
@@ -2005,17 +2005,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>34 (may be duplicate - check)</t>
+          <t>9 (Talk to Derek)</t>
         </is>
       </c>
       <c r="B84" t="b">
         <v>0</v>
       </c>
       <c r="C84" t="n">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="D84" t="n">
-        <v>96</v>
+        <v>95.94</v>
       </c>
       <c r="E84" t="n">
         <v>2</v>
@@ -2024,7 +2024,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>9 (Talk to Derek)</t>
+          <t>alter_layout</t>
         </is>
       </c>
       <c r="B85" t="b">
@@ -2043,17 +2043,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>alter_layout</t>
+          <t>drop_test</t>
         </is>
       </c>
       <c r="B86" t="b">
         <v>0</v>
       </c>
       <c r="C86" t="n">
-        <v>1750</v>
+        <v>1748</v>
       </c>
       <c r="D86" t="n">
-        <v>95.94</v>
+        <v>95.83</v>
       </c>
       <c r="E86" t="n">
         <v>2</v>
@@ -2062,17 +2062,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>drop_test</t>
+          <t>8 (62368-1 Dual)</t>
         </is>
       </c>
       <c r="B87" t="b">
         <v>0</v>
       </c>
       <c r="C87" t="n">
-        <v>1748</v>
+        <v>1747</v>
       </c>
       <c r="D87" t="n">
-        <v>95.83</v>
+        <v>95.78</v>
       </c>
       <c r="E87" t="n">
         <v>2</v>
@@ -2081,17 +2081,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>8 (62368-1 Dual)</t>
-        </is>
-      </c>
-      <c r="B88" t="b">
+          <t>type_of_investigation_2 - Full Investigation + Alternate Construction</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
         <v>0</v>
       </c>
       <c r="C88" t="n">
-        <v>1747</v>
+        <v>1744</v>
       </c>
       <c r="D88" t="n">
-        <v>95.78</v>
+        <v>95.61</v>
       </c>
       <c r="E88" t="n">
         <v>2</v>
@@ -2100,10 +2100,10 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>type_of_investigation_2 - Full Investigation + Alternate Construction</t>
-        </is>
-      </c>
-      <c r="B89" t="n">
+          <t>humidity_test</t>
+        </is>
+      </c>
+      <c r="B89" t="b">
         <v>0</v>
       </c>
       <c r="C89" t="n">
@@ -2119,17 +2119,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>humidity_test</t>
+          <t>working_voltage_test</t>
         </is>
       </c>
       <c r="B90" t="b">
         <v>0</v>
       </c>
       <c r="C90" t="n">
-        <v>1744</v>
+        <v>1742</v>
       </c>
       <c r="D90" t="n">
-        <v>95.61</v>
+        <v>95.5</v>
       </c>
       <c r="E90" t="n">
         <v>2</v>
@@ -2138,17 +2138,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>working_voltage_test</t>
-        </is>
-      </c>
-      <c r="B91" t="b">
+          <t>CCN_Top10_NWGQ</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
         <v>0</v>
       </c>
       <c r="C91" t="n">
-        <v>1742</v>
+        <v>1739</v>
       </c>
       <c r="D91" t="n">
-        <v>95.5</v>
+        <v>95.34</v>
       </c>
       <c r="E91" t="n">
         <v>2</v>
@@ -2157,17 +2157,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CCN_Top10_NWGQ</t>
+          <t>CCN_Top10_OTHER</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>0</v>
       </c>
       <c r="C92" t="n">
-        <v>1739</v>
+        <v>1736</v>
       </c>
       <c r="D92" t="n">
-        <v>95.34</v>
+        <v>95.18000000000001</v>
       </c>
       <c r="E92" t="n">
         <v>2</v>
@@ -2176,10 +2176,10 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CCN_Top10_OTHER</t>
-        </is>
-      </c>
-      <c r="B93" t="n">
+          <t>component_failure_test</t>
+        </is>
+      </c>
+      <c r="B93" t="b">
         <v>0</v>
       </c>
       <c r="C93" t="n">
@@ -2195,17 +2195,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>component_failure_test</t>
+          <t>SELV_reliability_test</t>
         </is>
       </c>
       <c r="B94" t="b">
         <v>0</v>
       </c>
       <c r="C94" t="n">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="D94" t="n">
-        <v>95.18000000000001</v>
+        <v>95.12</v>
       </c>
       <c r="E94" t="n">
         <v>2</v>
@@ -2214,11 +2214,11 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SELV_reliability_test</t>
+          <t>UL</t>
         </is>
       </c>
       <c r="B95" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C95" t="n">
         <v>1735</v>
@@ -2233,17 +2233,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>UL</t>
+          <t>cUL</t>
         </is>
       </c>
       <c r="B96" t="b">
         <v>1</v>
       </c>
       <c r="C96" t="n">
-        <v>1735</v>
+        <v>1733</v>
       </c>
       <c r="D96" t="n">
-        <v>95.12</v>
+        <v>95.01000000000001</v>
       </c>
       <c r="E96" t="n">
         <v>2</v>
@@ -2252,17 +2252,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>cUL</t>
+          <t>alter_fan</t>
         </is>
       </c>
       <c r="B97" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C97" t="n">
-        <v>1733</v>
+        <v>1730</v>
       </c>
       <c r="D97" t="n">
-        <v>95.01000000000001</v>
+        <v>94.84999999999999</v>
       </c>
       <c r="E97" t="n">
         <v>2</v>
@@ -2271,17 +2271,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>alter_fan</t>
+          <t>_60950_1_2ed_A2</t>
         </is>
       </c>
       <c r="B98" t="b">
         <v>0</v>
       </c>
       <c r="C98" t="n">
-        <v>1730</v>
+        <v>1717</v>
       </c>
       <c r="D98" t="n">
-        <v>94.84999999999999</v>
+        <v>94.13</v>
       </c>
       <c r="E98" t="n">
         <v>2</v>
@@ -2290,7 +2290,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>_60950_1_2ed_A2</t>
+          <t>11 (Ask Derek if  IEC/EN 62368-3  covers this)</t>
         </is>
       </c>
       <c r="B99" t="b">
@@ -2309,17 +2309,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>11 (Ask Derek if  IEC/EN 62368-3  covers this)</t>
+          <t>stalled_fan_test</t>
         </is>
       </c>
       <c r="B100" t="b">
         <v>0</v>
       </c>
       <c r="C100" t="n">
-        <v>1717</v>
+        <v>1716</v>
       </c>
       <c r="D100" t="n">
-        <v>94.13</v>
+        <v>94.08</v>
       </c>
       <c r="E100" t="n">
         <v>2</v>
@@ -2328,17 +2328,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>stalled_fan_test</t>
-        </is>
-      </c>
-      <c r="B101" t="b">
+          <t>CCN_Top10_QQJQ</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
         <v>0</v>
       </c>
       <c r="C101" t="n">
-        <v>1716</v>
+        <v>1701</v>
       </c>
       <c r="D101" t="n">
-        <v>94.08</v>
+        <v>93.26000000000001</v>
       </c>
       <c r="E101" t="n">
         <v>2</v>
@@ -2347,17 +2347,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CCN_Top10_QQJQ</t>
+          <t>CCN_Top10_QQJQ2</t>
         </is>
       </c>
       <c r="B102" t="n">
         <v>0</v>
       </c>
       <c r="C102" t="n">
-        <v>1701</v>
+        <v>1700</v>
       </c>
       <c r="D102" t="n">
-        <v>93.26000000000001</v>
+        <v>93.2</v>
       </c>
       <c r="E102" t="n">
         <v>2</v>
@@ -2366,17 +2366,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CCN_Top10_QQJQ2</t>
-        </is>
-      </c>
-      <c r="B103" t="n">
+          <t>blocked_vent_test</t>
+        </is>
+      </c>
+      <c r="B103" t="b">
         <v>0</v>
       </c>
       <c r="C103" t="n">
-        <v>1700</v>
+        <v>1698</v>
       </c>
       <c r="D103" t="n">
-        <v>93.2</v>
+        <v>93.09</v>
       </c>
       <c r="E103" t="n">
         <v>2</v>
@@ -2385,17 +2385,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>blocked_vent_test</t>
-        </is>
-      </c>
-      <c r="B104" t="b">
+          <t>1 (60950-1)</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
         <v>0</v>
       </c>
       <c r="C104" t="n">
-        <v>1698</v>
+        <v>1695</v>
       </c>
       <c r="D104" t="n">
-        <v>93.09</v>
+        <v>92.93000000000001</v>
       </c>
       <c r="E104" t="n">
         <v>2</v>
@@ -2404,17 +2404,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>1 (60950-1)</t>
+          <t>CCN_Top10_AZOT2</t>
         </is>
       </c>
       <c r="B105" t="n">
         <v>0</v>
       </c>
       <c r="C105" t="n">
-        <v>1695</v>
+        <v>1689</v>
       </c>
       <c r="D105" t="n">
-        <v>92.93000000000001</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="E105" t="n">
         <v>2</v>
@@ -2423,17 +2423,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>CCN_Top10_AZOT2</t>
-        </is>
-      </c>
-      <c r="B106" t="n">
+          <t>steady_force_test</t>
+        </is>
+      </c>
+      <c r="B106" t="b">
         <v>0</v>
       </c>
       <c r="C106" t="n">
-        <v>1689</v>
+        <v>1674</v>
       </c>
       <c r="D106" t="n">
-        <v>92.59999999999999</v>
+        <v>91.78</v>
       </c>
       <c r="E106" t="n">
         <v>2</v>
@@ -2442,17 +2442,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>steady_force_test</t>
+          <t>29 (Talk to Derek)</t>
         </is>
       </c>
       <c r="B107" t="b">
         <v>0</v>
       </c>
       <c r="C107" t="n">
-        <v>1674</v>
+        <v>1669</v>
       </c>
       <c r="D107" t="n">
-        <v>91.78</v>
+        <v>91.5</v>
       </c>
       <c r="E107" t="n">
         <v>2</v>
@@ -2461,17 +2461,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>29 (Talk to Derek)</t>
+          <t>capacitance_discharge_test</t>
         </is>
       </c>
       <c r="B108" t="b">
         <v>0</v>
       </c>
       <c r="C108" t="n">
-        <v>1669</v>
+        <v>1648</v>
       </c>
       <c r="D108" t="n">
-        <v>91.5</v>
+        <v>90.34999999999999</v>
       </c>
       <c r="E108" t="n">
         <v>2</v>
@@ -2480,38 +2480,19 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>capacitance_discharge_test</t>
+          <t>touch_current_single_test</t>
         </is>
       </c>
       <c r="B109" t="b">
         <v>0</v>
       </c>
       <c r="C109" t="n">
-        <v>1648</v>
+        <v>1644</v>
       </c>
       <c r="D109" t="n">
-        <v>90.34999999999999</v>
+        <v>90.13</v>
       </c>
       <c r="E109" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>touch_current_single_test</t>
-        </is>
-      </c>
-      <c r="B110" t="b">
-        <v>0</v>
-      </c>
-      <c r="C110" t="n">
-        <v>1644</v>
-      </c>
-      <c r="D110" t="n">
-        <v>90.13</v>
-      </c>
-      <c r="E110" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Morning 2/25 starting ML
</commit_message>
<xml_diff>
--- a/Code/1. Exploratory Data Analysis/near_constant_columns_90pct.xlsx
+++ b/Code/1. Exploratory Data Analysis/near_constant_columns_90pct.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E110"/>
+  <dimension ref="A1:E92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,93 +446,93 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3 (60950-21)</t>
+          <t>NOM</t>
         </is>
       </c>
       <c r="B2" t="b">
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>1824</v>
+        <v>1769</v>
       </c>
       <c r="D2" t="n">
-        <v>100</v>
+        <v>99.94</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>5 (60950-23)</t>
+          <t>PSE</t>
         </is>
       </c>
       <c r="B3" t="b">
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>1824</v>
+        <v>1769</v>
       </c>
       <c r="D3" t="n">
-        <v>100</v>
+        <v>99.94</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2 (EN 60950/EN 60065)</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="B4" t="b">
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>1824</v>
+        <v>1769</v>
       </c>
       <c r="D4" t="n">
-        <v>100</v>
+        <v>99.94</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BSMI</t>
+          <t>CCC</t>
         </is>
       </c>
       <c r="B5" t="b">
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>1824</v>
+        <v>1768</v>
       </c>
       <c r="D5" t="n">
-        <v>100</v>
+        <v>99.89</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NOM</t>
+          <t>thin_material_test</t>
         </is>
       </c>
       <c r="B6" t="b">
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>1823</v>
+        <v>1768</v>
       </c>
       <c r="D6" t="n">
-        <v>99.95</v>
+        <v>99.89</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -541,17 +541,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>Test- Bridging Resistor Test</t>
         </is>
       </c>
       <c r="B7" t="b">
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>1823</v>
+        <v>1768</v>
       </c>
       <c r="D7" t="n">
-        <v>99.95</v>
+        <v>99.89</v>
       </c>
       <c r="E7" t="n">
         <v>2</v>
@@ -560,17 +560,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PSE</t>
+          <t>102 (LFC)</t>
         </is>
       </c>
       <c r="B8" t="b">
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>1823</v>
+        <v>1767</v>
       </c>
       <c r="D8" t="n">
-        <v>99.95</v>
+        <v>99.83</v>
       </c>
       <c r="E8" t="n">
         <v>2</v>
@@ -579,17 +579,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>type_of_investigation_Missing</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+          <t>multilayer_boards</t>
+        </is>
+      </c>
+      <c r="B9" t="b">
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>1823</v>
+        <v>1767</v>
       </c>
       <c r="D9" t="n">
-        <v>99.95</v>
+        <v>99.83</v>
       </c>
       <c r="E9" t="n">
         <v>2</v>
@@ -598,17 +598,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CCC</t>
-        </is>
-      </c>
-      <c r="B10" t="b">
+          <t>total_schemmes</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>1822</v>
+        <v>1766</v>
       </c>
       <c r="D10" t="n">
-        <v>99.89</v>
+        <v>99.77</v>
       </c>
       <c r="E10" t="n">
         <v>2</v>
@@ -617,17 +617,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Test- Bridging Resistor Test</t>
+          <t>dust_test</t>
         </is>
       </c>
       <c r="B11" t="b">
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>1821</v>
+        <v>1766</v>
       </c>
       <c r="D11" t="n">
-        <v>99.84</v>
+        <v>99.77</v>
       </c>
       <c r="E11" t="n">
         <v>2</v>
@@ -636,17 +636,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>102 (LFC)</t>
+          <t>varistor_overload_test</t>
         </is>
       </c>
       <c r="B12" t="b">
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>1821</v>
+        <v>1766</v>
       </c>
       <c r="D12" t="n">
-        <v>99.84</v>
+        <v>99.77</v>
       </c>
       <c r="E12" t="n">
         <v>2</v>
@@ -655,17 +655,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>thin_material_test</t>
+          <t>alter_relay</t>
         </is>
       </c>
       <c r="B13" t="b">
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>1821</v>
+        <v>1764</v>
       </c>
       <c r="D13" t="n">
-        <v>99.84</v>
+        <v>99.66</v>
       </c>
       <c r="E13" t="n">
         <v>2</v>
@@ -674,17 +674,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>multilayer_boards</t>
+          <t>103 (L R Over DC Mot in Sec Cir)</t>
         </is>
       </c>
       <c r="B14" t="b">
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>1821</v>
+        <v>1763</v>
       </c>
       <c r="D14" t="n">
-        <v>99.84</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="E14" t="n">
         <v>2</v>
@@ -693,17 +693,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>varistor_overload_test</t>
+          <t>uncertified_pwr_supply</t>
         </is>
       </c>
       <c r="B15" t="b">
         <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>1820</v>
+        <v>1763</v>
       </c>
       <c r="D15" t="n">
-        <v>99.78</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="E15" t="n">
         <v>2</v>
@@ -712,17 +712,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>total_schemmes</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+          <t>unknown_PWR_supply</t>
+        </is>
+      </c>
+      <c r="B16" t="b">
         <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>1820</v>
+        <v>1763</v>
       </c>
       <c r="D16" t="n">
-        <v>99.78</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="E16" t="n">
         <v>2</v>
@@ -731,17 +731,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>dust_test</t>
+          <t>energy_hazard_test</t>
         </is>
       </c>
       <c r="B17" t="b">
         <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>1819</v>
+        <v>1763</v>
       </c>
       <c r="D17" t="n">
-        <v>99.73</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="E17" t="n">
         <v>2</v>
@@ -750,17 +750,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>unknown_PWR_supply</t>
+          <t>alter_interconnect</t>
         </is>
       </c>
       <c r="B18" t="b">
         <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>1817</v>
+        <v>1763</v>
       </c>
       <c r="D18" t="n">
-        <v>99.62</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="E18" t="n">
         <v>2</v>
@@ -769,17 +769,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>uncertified_pwr_supply</t>
+          <t>moment_test</t>
         </is>
       </c>
       <c r="B19" t="b">
         <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>1817</v>
+        <v>1762</v>
       </c>
       <c r="D19" t="n">
-        <v>99.62</v>
+        <v>99.55</v>
       </c>
       <c r="E19" t="n">
         <v>2</v>
@@ -788,17 +788,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>103 (L R Over DC Mot in Sec Cir)</t>
+          <t>alter_strain_relief</t>
         </is>
       </c>
       <c r="B20" t="b">
         <v>0</v>
       </c>
       <c r="C20" t="n">
-        <v>1816</v>
+        <v>1762</v>
       </c>
       <c r="D20" t="n">
-        <v>99.56</v>
+        <v>99.55</v>
       </c>
       <c r="E20" t="n">
         <v>2</v>
@@ -807,17 +807,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>energy_hazard_test</t>
-        </is>
-      </c>
-      <c r="B21" t="b">
+          <t>CCN_Top10_NWIN</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
         <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>1816</v>
+        <v>1761</v>
       </c>
       <c r="D21" t="n">
-        <v>99.56</v>
+        <v>99.48999999999999</v>
       </c>
       <c r="E21" t="n">
         <v>2</v>
@@ -826,17 +826,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>moment_test</t>
+          <t>Test- Secondary Working Voltage</t>
         </is>
       </c>
       <c r="B22" t="b">
         <v>0</v>
       </c>
       <c r="C22" t="n">
-        <v>1815</v>
+        <v>1761</v>
       </c>
       <c r="D22" t="n">
-        <v>99.51000000000001</v>
+        <v>99.48999999999999</v>
       </c>
       <c r="E22" t="n">
         <v>2</v>
@@ -845,17 +845,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CCN_Top10_NWIN</t>
+          <t>Investigation_type_4 - DC Distribution Panels</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>1815</v>
+        <v>1761</v>
       </c>
       <c r="D23" t="n">
-        <v>99.51000000000001</v>
+        <v>99.48999999999999</v>
       </c>
       <c r="E23" t="n">
         <v>2</v>
@@ -864,17 +864,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>alter_strain_relief</t>
+          <t>outdoor_use</t>
         </is>
       </c>
       <c r="B24" t="b">
         <v>0</v>
       </c>
       <c r="C24" t="n">
-        <v>1815</v>
+        <v>1760</v>
       </c>
       <c r="D24" t="n">
-        <v>99.51000000000001</v>
+        <v>99.44</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -883,17 +883,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>alter_interconnect</t>
+          <t>alter_cord</t>
         </is>
       </c>
       <c r="B25" t="b">
         <v>0</v>
       </c>
       <c r="C25" t="n">
-        <v>1815</v>
+        <v>1759</v>
       </c>
       <c r="D25" t="n">
-        <v>99.51000000000001</v>
+        <v>99.38</v>
       </c>
       <c r="E25" t="n">
         <v>2</v>
@@ -902,17 +902,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>alter_relay</t>
+          <t>alter_resistor</t>
         </is>
       </c>
       <c r="B26" t="b">
         <v>0</v>
       </c>
       <c r="C26" t="n">
-        <v>1815</v>
+        <v>1759</v>
       </c>
       <c r="D26" t="n">
-        <v>99.51000000000001</v>
+        <v>99.38</v>
       </c>
       <c r="E26" t="n">
         <v>2</v>
@@ -921,17 +921,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Test- Secondary Working Voltage</t>
+          <t>PoE_source</t>
         </is>
       </c>
       <c r="B27" t="b">
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>1815</v>
+        <v>1759</v>
       </c>
       <c r="D27" t="n">
-        <v>99.51000000000001</v>
+        <v>99.38</v>
       </c>
       <c r="E27" t="n">
         <v>2</v>
@@ -940,17 +940,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Investigation_type_4 - DC Distribution Panels</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
+          <t>7 (950 TO 368)</t>
+        </is>
+      </c>
+      <c r="B28" t="b">
         <v>0</v>
       </c>
       <c r="C28" t="n">
-        <v>1814</v>
+        <v>1759</v>
       </c>
       <c r="D28" t="n">
-        <v>99.45</v>
+        <v>99.38</v>
       </c>
       <c r="E28" t="n">
         <v>2</v>
@@ -959,17 +959,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>outdoor_use</t>
+          <t>Test- Tensile Strength</t>
         </is>
       </c>
       <c r="B29" t="b">
         <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>1814</v>
+        <v>1759</v>
       </c>
       <c r="D29" t="n">
-        <v>99.45</v>
+        <v>99.38</v>
       </c>
       <c r="E29" t="n">
         <v>2</v>
@@ -978,17 +978,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Test- Tensile Strength</t>
+          <t>alter_movs</t>
         </is>
       </c>
       <c r="B30" t="b">
         <v>0</v>
       </c>
       <c r="C30" t="n">
-        <v>1813</v>
+        <v>1758</v>
       </c>
       <c r="D30" t="n">
-        <v>99.40000000000001</v>
+        <v>99.31999999999999</v>
       </c>
       <c r="E30" t="n">
         <v>2</v>
@@ -997,17 +997,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>alter_cord</t>
+          <t>alter_app_inlet</t>
         </is>
       </c>
       <c r="B31" t="b">
         <v>0</v>
       </c>
       <c r="C31" t="n">
-        <v>1813</v>
+        <v>1758</v>
       </c>
       <c r="D31" t="n">
-        <v>99.40000000000001</v>
+        <v>99.31999999999999</v>
       </c>
       <c r="E31" t="n">
         <v>2</v>
@@ -1016,17 +1016,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>PoE_source</t>
-        </is>
-      </c>
-      <c r="B32" t="b">
+          <t>type_of_investigation_5 - Administrative CB review</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
         <v>0</v>
       </c>
       <c r="C32" t="n">
-        <v>1813</v>
+        <v>1757</v>
       </c>
       <c r="D32" t="n">
-        <v>99.40000000000001</v>
+        <v>99.27</v>
       </c>
       <c r="E32" t="n">
         <v>2</v>
@@ -1035,17 +1035,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7 (950 TO 368)</t>
+          <t>all_mount_test</t>
         </is>
       </c>
       <c r="B33" t="b">
         <v>0</v>
       </c>
       <c r="C33" t="n">
-        <v>1812</v>
+        <v>1756</v>
       </c>
       <c r="D33" t="n">
-        <v>99.34</v>
+        <v>99.20999999999999</v>
       </c>
       <c r="E33" t="n">
         <v>2</v>
@@ -1054,17 +1054,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>alter_movs</t>
-        </is>
-      </c>
-      <c r="B34" t="b">
+          <t>CCN_Top10_QQGQ2</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
         <v>0</v>
       </c>
       <c r="C34" t="n">
-        <v>1811</v>
+        <v>1756</v>
       </c>
       <c r="D34" t="n">
-        <v>99.29000000000001</v>
+        <v>99.20999999999999</v>
       </c>
       <c r="E34" t="n">
         <v>2</v>
@@ -1073,17 +1073,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>alter_app_inlet</t>
+          <t>strain_relief_test</t>
         </is>
       </c>
       <c r="B35" t="b">
         <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>1811</v>
+        <v>1755</v>
       </c>
       <c r="D35" t="n">
-        <v>99.29000000000001</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="E35" t="n">
         <v>2</v>
@@ -1092,17 +1092,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>type_of_investigation_5 - Administrative CB review</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
+          <t>alter_LPS</t>
+        </is>
+      </c>
+      <c r="B36" t="b">
         <v>0</v>
       </c>
       <c r="C36" t="n">
-        <v>1811</v>
+        <v>1755</v>
       </c>
       <c r="D36" t="n">
-        <v>99.29000000000001</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="E36" t="n">
         <v>2</v>
@@ -1111,17 +1111,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>alter_resistor</t>
+          <t>alter_display</t>
         </is>
       </c>
       <c r="B37" t="b">
         <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>1810</v>
+        <v>1755</v>
       </c>
       <c r="D37" t="n">
-        <v>99.23</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="E37" t="n">
         <v>2</v>
@@ -1130,17 +1130,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>all_mount_test</t>
+          <t>touch_current_test</t>
         </is>
       </c>
       <c r="B38" t="b">
         <v>0</v>
       </c>
       <c r="C38" t="n">
-        <v>1810</v>
+        <v>1755</v>
       </c>
       <c r="D38" t="n">
-        <v>99.23</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="E38" t="n">
         <v>2</v>
@@ -1149,17 +1149,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>alter_LPS</t>
+          <t>alter_light</t>
         </is>
       </c>
       <c r="B39" t="b">
         <v>0</v>
       </c>
       <c r="C39" t="n">
-        <v>1809</v>
+        <v>1754</v>
       </c>
       <c r="D39" t="n">
-        <v>99.18000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="E39" t="n">
         <v>2</v>
@@ -1168,17 +1168,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CCN_Top10_QQGQ2</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
+          <t>preliminary_review</t>
+        </is>
+      </c>
+      <c r="B40" t="b">
         <v>0</v>
       </c>
       <c r="C40" t="n">
-        <v>1809</v>
+        <v>1754</v>
       </c>
       <c r="D40" t="n">
-        <v>99.18000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="E40" t="n">
         <v>2</v>
@@ -1187,17 +1187,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>strain_relief_test</t>
+          <t>alter_ptc</t>
         </is>
       </c>
       <c r="B41" t="b">
         <v>0</v>
       </c>
       <c r="C41" t="n">
-        <v>1809</v>
+        <v>1754</v>
       </c>
       <c r="D41" t="n">
-        <v>99.18000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="E41" t="n">
         <v>2</v>
@@ -1206,17 +1206,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>alter_display</t>
+          <t>water_spray_test</t>
         </is>
       </c>
       <c r="B42" t="b">
         <v>0</v>
       </c>
       <c r="C42" t="n">
-        <v>1809</v>
+        <v>1753</v>
       </c>
       <c r="D42" t="n">
-        <v>99.18000000000001</v>
+        <v>99.04000000000001</v>
       </c>
       <c r="E42" t="n">
         <v>2</v>
@@ -1225,17 +1225,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>alter_ptc</t>
+          <t>alter_optical_isolator</t>
         </is>
       </c>
       <c r="B43" t="b">
         <v>0</v>
       </c>
       <c r="C43" t="n">
-        <v>1808</v>
+        <v>1753</v>
       </c>
       <c r="D43" t="n">
-        <v>99.12</v>
+        <v>99.04000000000001</v>
       </c>
       <c r="E43" t="n">
         <v>2</v>
@@ -1244,17 +1244,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>alter_light</t>
+          <t>stability_test</t>
         </is>
       </c>
       <c r="B44" t="b">
         <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>1808</v>
+        <v>1753</v>
       </c>
       <c r="D44" t="n">
-        <v>99.12</v>
+        <v>99.04000000000001</v>
       </c>
       <c r="E44" t="n">
         <v>2</v>
@@ -1263,17 +1263,18 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>preliminary_review</t>
+          <t xml:space="preserve">
+33 (Rename)</t>
         </is>
       </c>
       <c r="B45" t="b">
         <v>0</v>
       </c>
       <c r="C45" t="n">
-        <v>1807</v>
+        <v>1752</v>
       </c>
       <c r="D45" t="n">
-        <v>99.06999999999999</v>
+        <v>98.98</v>
       </c>
       <c r="E45" t="n">
         <v>2</v>
@@ -1282,17 +1283,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>touch_current_test</t>
+          <t>PoE_load</t>
         </is>
       </c>
       <c r="B46" t="b">
         <v>0</v>
       </c>
       <c r="C46" t="n">
-        <v>1807</v>
+        <v>1751</v>
       </c>
       <c r="D46" t="n">
-        <v>99.06999999999999</v>
+        <v>98.93000000000001</v>
       </c>
       <c r="E46" t="n">
         <v>2</v>
@@ -1301,17 +1302,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>water_spray_test</t>
-        </is>
-      </c>
-      <c r="B47" t="b">
+          <t>CCN_Top10_AAAL</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
         <v>0</v>
       </c>
       <c r="C47" t="n">
-        <v>1807</v>
+        <v>1751</v>
       </c>
       <c r="D47" t="n">
-        <v>99.06999999999999</v>
+        <v>98.93000000000001</v>
       </c>
       <c r="E47" t="n">
         <v>2</v>
@@ -1320,17 +1321,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>stability_test</t>
+          <t>_60950_1_62368_1_2nd-3rd_CheckBox</t>
         </is>
       </c>
       <c r="B48" t="b">
         <v>0</v>
       </c>
       <c r="C48" t="n">
-        <v>1807</v>
+        <v>1750</v>
       </c>
       <c r="D48" t="n">
-        <v>99.06999999999999</v>
+        <v>98.87</v>
       </c>
       <c r="E48" t="n">
         <v>2</v>
@@ -1339,17 +1340,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>alter_optical_isolator</t>
+          <t>family_grouping</t>
         </is>
       </c>
       <c r="B49" t="b">
         <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>1806</v>
+        <v>1750</v>
       </c>
       <c r="D49" t="n">
-        <v>99.01000000000001</v>
+        <v>98.87</v>
       </c>
       <c r="E49" t="n">
         <v>2</v>
@@ -1358,17 +1359,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PoE_load</t>
+          <t>alter_fuse</t>
         </is>
       </c>
       <c r="B50" t="b">
         <v>0</v>
       </c>
       <c r="C50" t="n">
-        <v>1805</v>
+        <v>1747</v>
       </c>
       <c r="D50" t="n">
-        <v>98.95999999999999</v>
+        <v>98.7</v>
       </c>
       <c r="E50" t="n">
         <v>2</v>
@@ -1377,17 +1378,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>_60950_1_62368_1_2nd-3rd_CheckBox</t>
+          <t>alter_complex</t>
         </is>
       </c>
       <c r="B51" t="b">
         <v>0</v>
       </c>
       <c r="C51" t="n">
-        <v>1804</v>
+        <v>1745</v>
       </c>
       <c r="D51" t="n">
-        <v>98.90000000000001</v>
+        <v>98.59</v>
       </c>
       <c r="E51" t="n">
         <v>2</v>
@@ -1396,17 +1397,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CCN_Top10_AAAL</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
+          <t>4 (Annex Y)</t>
+        </is>
+      </c>
+      <c r="B52" t="b">
         <v>0</v>
       </c>
       <c r="C52" t="n">
-        <v>1804</v>
+        <v>1745</v>
       </c>
       <c r="D52" t="n">
-        <v>98.90000000000001</v>
+        <v>98.59</v>
       </c>
       <c r="E52" t="n">
         <v>2</v>
@@ -1415,18 +1416,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">
-33 (Rename)</t>
+          <t>alter_inductor</t>
         </is>
       </c>
       <c r="B53" t="b">
         <v>0</v>
       </c>
       <c r="C53" t="n">
-        <v>1802</v>
+        <v>1745</v>
       </c>
       <c r="D53" t="n">
-        <v>98.79000000000001</v>
+        <v>98.59</v>
       </c>
       <c r="E53" t="n">
         <v>2</v>
@@ -1435,17 +1435,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>alter_fuse</t>
+          <t>power_measurement_test</t>
         </is>
       </c>
       <c r="B54" t="b">
         <v>0</v>
       </c>
       <c r="C54" t="n">
-        <v>1800</v>
+        <v>1744</v>
       </c>
       <c r="D54" t="n">
-        <v>98.68000000000001</v>
+        <v>98.53</v>
       </c>
       <c r="E54" t="n">
         <v>2</v>
@@ -1454,17 +1454,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>alter_complex</t>
-        </is>
-      </c>
-      <c r="B55" t="b">
+          <t>CCN_Top10_AALL</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
         <v>0</v>
       </c>
       <c r="C55" t="n">
-        <v>1799</v>
+        <v>1742</v>
       </c>
       <c r="D55" t="n">
-        <v>98.63</v>
+        <v>98.42</v>
       </c>
       <c r="E55" t="n">
         <v>2</v>
@@ -1473,17 +1473,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>alter_inductor</t>
+          <t>alter_connector</t>
         </is>
       </c>
       <c r="B56" t="b">
         <v>0</v>
       </c>
       <c r="C56" t="n">
-        <v>1797</v>
+        <v>1742</v>
       </c>
       <c r="D56" t="n">
-        <v>98.52</v>
+        <v>98.42</v>
       </c>
       <c r="E56" t="n">
         <v>2</v>
@@ -1492,17 +1492,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>family_grouping</t>
-        </is>
-      </c>
-      <c r="B57" t="b">
+          <t>CCN_Top10_AAAU</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
         <v>0</v>
       </c>
       <c r="C57" t="n">
-        <v>1797</v>
+        <v>1742</v>
       </c>
       <c r="D57" t="n">
-        <v>98.52</v>
+        <v>98.42</v>
       </c>
       <c r="E57" t="n">
         <v>2</v>
@@ -1511,17 +1511,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>power_measurement_test</t>
+          <t>alter_transformer</t>
         </is>
       </c>
       <c r="B58" t="b">
         <v>0</v>
       </c>
       <c r="C58" t="n">
-        <v>1796</v>
+        <v>1738</v>
       </c>
       <c r="D58" t="n">
-        <v>98.45999999999999</v>
+        <v>98.19</v>
       </c>
       <c r="E58" t="n">
         <v>2</v>
@@ -1530,17 +1530,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>4 (Annex Y)</t>
+          <t>ball_pressue_test</t>
         </is>
       </c>
       <c r="B59" t="b">
         <v>0</v>
       </c>
       <c r="C59" t="n">
-        <v>1795</v>
+        <v>1736</v>
       </c>
       <c r="D59" t="n">
-        <v>98.41</v>
+        <v>98.08</v>
       </c>
       <c r="E59" t="n">
         <v>2</v>
@@ -1549,17 +1549,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>alter_connector</t>
+          <t>batteries_present</t>
         </is>
       </c>
       <c r="B60" t="b">
         <v>0</v>
       </c>
       <c r="C60" t="n">
-        <v>1795</v>
+        <v>1736</v>
       </c>
       <c r="D60" t="n">
-        <v>98.41</v>
+        <v>98.08</v>
       </c>
       <c r="E60" t="n">
         <v>2</v>
@@ -1568,17 +1568,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CCN_Top10_AAAU</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
+          <t>IT Informational Test Report</t>
+        </is>
+      </c>
+      <c r="B61" t="b">
         <v>0</v>
       </c>
       <c r="C61" t="n">
-        <v>1794</v>
+        <v>1735</v>
       </c>
       <c r="D61" t="n">
-        <v>98.36</v>
+        <v>98.02</v>
       </c>
       <c r="E61" t="n">
         <v>2</v>
@@ -1587,17 +1587,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>batteries_present</t>
+          <t>loading_wall_test</t>
         </is>
       </c>
       <c r="B62" t="b">
         <v>0</v>
       </c>
       <c r="C62" t="n">
-        <v>1790</v>
+        <v>1733</v>
       </c>
       <c r="D62" t="n">
-        <v>98.14</v>
+        <v>97.91</v>
       </c>
       <c r="E62" t="n">
         <v>2</v>
@@ -1606,17 +1606,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CCN_Top10_AALL</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
+          <t>batt_drop_test</t>
+        </is>
+      </c>
+      <c r="B63" t="b">
         <v>0</v>
       </c>
       <c r="C63" t="n">
-        <v>1790</v>
+        <v>1732</v>
       </c>
       <c r="D63" t="n">
-        <v>98.14</v>
+        <v>97.84999999999999</v>
       </c>
       <c r="E63" t="n">
         <v>2</v>
@@ -1625,17 +1625,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>alter_transformer</t>
+          <t>protective_bondingII_test</t>
         </is>
       </c>
       <c r="B64" t="b">
         <v>0</v>
       </c>
       <c r="C64" t="n">
-        <v>1789</v>
+        <v>1731</v>
       </c>
       <c r="D64" t="n">
-        <v>98.08</v>
+        <v>97.8</v>
       </c>
       <c r="E64" t="n">
         <v>2</v>
@@ -1644,17 +1644,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>IT Informational Test Report</t>
+          <t>30 (Talk to Derek)</t>
         </is>
       </c>
       <c r="B65" t="b">
         <v>0</v>
       </c>
       <c r="C65" t="n">
-        <v>1788</v>
+        <v>1731</v>
       </c>
       <c r="D65" t="n">
-        <v>98.03</v>
+        <v>97.8</v>
       </c>
       <c r="E65" t="n">
         <v>2</v>
@@ -1663,17 +1663,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>loading_wall_test</t>
+          <t>alter_insulation</t>
         </is>
       </c>
       <c r="B66" t="b">
         <v>0</v>
       </c>
       <c r="C66" t="n">
-        <v>1787</v>
+        <v>1731</v>
       </c>
       <c r="D66" t="n">
-        <v>97.97</v>
+        <v>97.8</v>
       </c>
       <c r="E66" t="n">
         <v>2</v>
@@ -1682,17 +1682,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ball_pressue_test</t>
+          <t>XFR_abnormal_operation_test</t>
         </is>
       </c>
       <c r="B67" t="b">
         <v>0</v>
       </c>
       <c r="C67" t="n">
-        <v>1786</v>
+        <v>1731</v>
       </c>
       <c r="D67" t="n">
-        <v>97.92</v>
+        <v>97.8</v>
       </c>
       <c r="E67" t="n">
         <v>2</v>
@@ -1701,17 +1701,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>batt_drop_test</t>
+          <t>max_output_test</t>
         </is>
       </c>
       <c r="B68" t="b">
         <v>0</v>
       </c>
       <c r="C68" t="n">
-        <v>1786</v>
+        <v>1729</v>
       </c>
       <c r="D68" t="n">
-        <v>97.92</v>
+        <v>97.68000000000001</v>
       </c>
       <c r="E68" t="n">
         <v>2</v>
@@ -1720,17 +1720,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>XFR_abnormal_operation_test</t>
+          <t>alter_capacitor</t>
         </is>
       </c>
       <c r="B69" t="b">
         <v>0</v>
       </c>
       <c r="C69" t="n">
-        <v>1783</v>
+        <v>1727</v>
       </c>
       <c r="D69" t="n">
-        <v>97.75</v>
+        <v>97.56999999999999</v>
       </c>
       <c r="E69" t="n">
         <v>2</v>
@@ -1739,17 +1739,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>protective_bondingII_test</t>
+          <t>enclosure_push_test</t>
         </is>
       </c>
       <c r="B70" t="b">
         <v>0</v>
       </c>
       <c r="C70" t="n">
-        <v>1783</v>
+        <v>1727</v>
       </c>
       <c r="D70" t="n">
-        <v>97.75</v>
+        <v>97.56999999999999</v>
       </c>
       <c r="E70" t="n">
         <v>2</v>
@@ -1758,17 +1758,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>alter_insulation</t>
+          <t>Test- Secondary Lithium Charge</t>
         </is>
       </c>
       <c r="B71" t="b">
         <v>0</v>
       </c>
       <c r="C71" t="n">
-        <v>1782</v>
+        <v>1725</v>
       </c>
       <c r="D71" t="n">
-        <v>97.7</v>
+        <v>97.45999999999999</v>
       </c>
       <c r="E71" t="n">
         <v>2</v>
@@ -1777,17 +1777,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>max_output_test</t>
+          <t>alter_current_ic</t>
         </is>
       </c>
       <c r="B72" t="b">
         <v>0</v>
       </c>
       <c r="C72" t="n">
-        <v>1782</v>
+        <v>1724</v>
       </c>
       <c r="D72" t="n">
-        <v>97.7</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="E72" t="n">
         <v>2</v>
@@ -1796,17 +1796,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>alter_capacitor</t>
+          <t>XFR_strength_test</t>
         </is>
       </c>
       <c r="B73" t="b">
         <v>0</v>
       </c>
       <c r="C73" t="n">
-        <v>1780</v>
+        <v>1722</v>
       </c>
       <c r="D73" t="n">
-        <v>97.59</v>
+        <v>97.29000000000001</v>
       </c>
       <c r="E73" t="n">
         <v>2</v>
@@ -1815,17 +1815,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Test- Secondary Lithium Charge</t>
+          <t>LCC_test</t>
         </is>
       </c>
       <c r="B74" t="b">
         <v>0</v>
       </c>
       <c r="C74" t="n">
-        <v>1779</v>
+        <v>1720</v>
       </c>
       <c r="D74" t="n">
-        <v>97.53</v>
+        <v>97.18000000000001</v>
       </c>
       <c r="E74" t="n">
         <v>2</v>
@@ -1834,17 +1834,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>enclosure_push_test</t>
+          <t>CB_reissue</t>
         </is>
       </c>
       <c r="B75" t="b">
         <v>0</v>
       </c>
       <c r="C75" t="n">
-        <v>1779</v>
+        <v>1720</v>
       </c>
       <c r="D75" t="n">
-        <v>97.53</v>
+        <v>97.18000000000001</v>
       </c>
       <c r="E75" t="n">
         <v>2</v>
@@ -1853,17 +1853,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>alter_current_ic</t>
+          <t>34 (may be duplicate - check)</t>
         </is>
       </c>
       <c r="B76" t="b">
         <v>0</v>
       </c>
       <c r="C76" t="n">
-        <v>1778</v>
+        <v>1715</v>
       </c>
       <c r="D76" t="n">
-        <v>97.48</v>
+        <v>96.89</v>
       </c>
       <c r="E76" t="n">
         <v>2</v>
@@ -1872,17 +1872,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>30 (Talk to Derek)</t>
+          <t>PS_shortcircuit_test</t>
         </is>
       </c>
       <c r="B77" t="b">
         <v>0</v>
       </c>
       <c r="C77" t="n">
-        <v>1774</v>
+        <v>1707</v>
       </c>
       <c r="D77" t="n">
-        <v>97.26000000000001</v>
+        <v>96.44</v>
       </c>
       <c r="E77" t="n">
         <v>2</v>
@@ -1891,17 +1891,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>LCC_test</t>
+          <t>alter_layout</t>
         </is>
       </c>
       <c r="B78" t="b">
         <v>0</v>
       </c>
       <c r="C78" t="n">
-        <v>1773</v>
+        <v>1700</v>
       </c>
       <c r="D78" t="n">
-        <v>97.2</v>
+        <v>96.05</v>
       </c>
       <c r="E78" t="n">
         <v>2</v>
@@ -1910,17 +1910,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CB_reissue</t>
+          <t>pro_bond_test</t>
         </is>
       </c>
       <c r="B79" t="b">
         <v>0</v>
       </c>
       <c r="C79" t="n">
-        <v>1772</v>
+        <v>1699</v>
       </c>
       <c r="D79" t="n">
-        <v>97.15000000000001</v>
+        <v>95.98999999999999</v>
       </c>
       <c r="E79" t="n">
         <v>2</v>
@@ -1929,17 +1929,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>XFR_strength_test</t>
+          <t>Test- Battery Protection Circuit</t>
         </is>
       </c>
       <c r="B80" t="b">
         <v>0</v>
       </c>
       <c r="C80" t="n">
-        <v>1772</v>
+        <v>1697</v>
       </c>
       <c r="D80" t="n">
-        <v>97.15000000000001</v>
+        <v>95.88</v>
       </c>
       <c r="E80" t="n">
         <v>2</v>
@@ -1948,17 +1948,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>PS_shortcircuit_test</t>
-        </is>
-      </c>
-      <c r="B81" t="b">
+          <t>CCN_Top10_NWGQ</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
         <v>0</v>
       </c>
       <c r="C81" t="n">
-        <v>1759</v>
+        <v>1697</v>
       </c>
       <c r="D81" t="n">
-        <v>96.44</v>
+        <v>95.88</v>
       </c>
       <c r="E81" t="n">
         <v>2</v>
@@ -1967,17 +1967,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>pro_bond_test</t>
+          <t>9 (Talk to Derek)</t>
         </is>
       </c>
       <c r="B82" t="b">
         <v>0</v>
       </c>
       <c r="C82" t="n">
-        <v>1751</v>
+        <v>1697</v>
       </c>
       <c r="D82" t="n">
-        <v>96</v>
+        <v>95.88</v>
       </c>
       <c r="E82" t="n">
         <v>2</v>
@@ -1986,17 +1986,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Test- Battery Protection Circuit</t>
+          <t>8 (62368-1 Dual)</t>
         </is>
       </c>
       <c r="B83" t="b">
         <v>0</v>
       </c>
       <c r="C83" t="n">
-        <v>1751</v>
+        <v>1695</v>
       </c>
       <c r="D83" t="n">
-        <v>96</v>
+        <v>95.76000000000001</v>
       </c>
       <c r="E83" t="n">
         <v>2</v>
@@ -2005,17 +2005,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>34 (may be duplicate - check)</t>
+          <t>drop_test</t>
         </is>
       </c>
       <c r="B84" t="b">
         <v>0</v>
       </c>
       <c r="C84" t="n">
-        <v>1751</v>
+        <v>1695</v>
       </c>
       <c r="D84" t="n">
-        <v>96</v>
+        <v>95.76000000000001</v>
       </c>
       <c r="E84" t="n">
         <v>2</v>
@@ -2024,17 +2024,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>9 (Talk to Derek)</t>
-        </is>
-      </c>
-      <c r="B85" t="b">
+          <t>type_of_investigation_2 - Full Investigation + Alternate Construction</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
         <v>0</v>
       </c>
       <c r="C85" t="n">
-        <v>1750</v>
+        <v>1691</v>
       </c>
       <c r="D85" t="n">
-        <v>95.94</v>
+        <v>95.54000000000001</v>
       </c>
       <c r="E85" t="n">
         <v>2</v>
@@ -2043,17 +2043,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>alter_layout</t>
+          <t>humidity_test</t>
         </is>
       </c>
       <c r="B86" t="b">
         <v>0</v>
       </c>
       <c r="C86" t="n">
-        <v>1750</v>
+        <v>1691</v>
       </c>
       <c r="D86" t="n">
-        <v>95.94</v>
+        <v>95.54000000000001</v>
       </c>
       <c r="E86" t="n">
         <v>2</v>
@@ -2062,17 +2062,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>drop_test</t>
-        </is>
-      </c>
-      <c r="B87" t="b">
+          <t>CCN_Top10_OTHER</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
         <v>0</v>
       </c>
       <c r="C87" t="n">
-        <v>1748</v>
+        <v>1691</v>
       </c>
       <c r="D87" t="n">
-        <v>95.83</v>
+        <v>95.54000000000001</v>
       </c>
       <c r="E87" t="n">
         <v>2</v>
@@ -2081,17 +2081,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>8 (62368-1 Dual)</t>
+          <t>working_voltage_test</t>
         </is>
       </c>
       <c r="B88" t="b">
         <v>0</v>
       </c>
       <c r="C88" t="n">
-        <v>1747</v>
+        <v>1689</v>
       </c>
       <c r="D88" t="n">
-        <v>95.78</v>
+        <v>95.42</v>
       </c>
       <c r="E88" t="n">
         <v>2</v>
@@ -2100,17 +2100,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>type_of_investigation_2 - Full Investigation + Alternate Construction</t>
-        </is>
-      </c>
-      <c r="B89" t="n">
-        <v>0</v>
+          <t>UL</t>
+        </is>
+      </c>
+      <c r="B89" t="b">
+        <v>1</v>
       </c>
       <c r="C89" t="n">
-        <v>1744</v>
+        <v>1688</v>
       </c>
       <c r="D89" t="n">
-        <v>95.61</v>
+        <v>95.37</v>
       </c>
       <c r="E89" t="n">
         <v>2</v>
@@ -2119,17 +2119,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>humidity_test</t>
+          <t>cUL</t>
         </is>
       </c>
       <c r="B90" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C90" t="n">
-        <v>1744</v>
+        <v>1686</v>
       </c>
       <c r="D90" t="n">
-        <v>95.61</v>
+        <v>95.25</v>
       </c>
       <c r="E90" t="n">
         <v>2</v>
@@ -2138,17 +2138,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>working_voltage_test</t>
+          <t>component_failure_test</t>
         </is>
       </c>
       <c r="B91" t="b">
         <v>0</v>
       </c>
       <c r="C91" t="n">
-        <v>1742</v>
+        <v>1684</v>
       </c>
       <c r="D91" t="n">
-        <v>95.5</v>
+        <v>95.14</v>
       </c>
       <c r="E91" t="n">
         <v>2</v>
@@ -2157,361 +2157,19 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CCN_Top10_NWGQ</t>
-        </is>
-      </c>
-      <c r="B92" t="n">
+          <t>SELV_reliability_test</t>
+        </is>
+      </c>
+      <c r="B92" t="b">
         <v>0</v>
       </c>
       <c r="C92" t="n">
-        <v>1739</v>
+        <v>1683</v>
       </c>
       <c r="D92" t="n">
-        <v>95.34</v>
+        <v>95.08</v>
       </c>
       <c r="E92" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>CCN_Top10_OTHER</t>
-        </is>
-      </c>
-      <c r="B93" t="n">
-        <v>0</v>
-      </c>
-      <c r="C93" t="n">
-        <v>1736</v>
-      </c>
-      <c r="D93" t="n">
-        <v>95.18000000000001</v>
-      </c>
-      <c r="E93" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>component_failure_test</t>
-        </is>
-      </c>
-      <c r="B94" t="b">
-        <v>0</v>
-      </c>
-      <c r="C94" t="n">
-        <v>1736</v>
-      </c>
-      <c r="D94" t="n">
-        <v>95.18000000000001</v>
-      </c>
-      <c r="E94" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>SELV_reliability_test</t>
-        </is>
-      </c>
-      <c r="B95" t="b">
-        <v>0</v>
-      </c>
-      <c r="C95" t="n">
-        <v>1735</v>
-      </c>
-      <c r="D95" t="n">
-        <v>95.12</v>
-      </c>
-      <c r="E95" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>UL</t>
-        </is>
-      </c>
-      <c r="B96" t="b">
-        <v>1</v>
-      </c>
-      <c r="C96" t="n">
-        <v>1735</v>
-      </c>
-      <c r="D96" t="n">
-        <v>95.12</v>
-      </c>
-      <c r="E96" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>cUL</t>
-        </is>
-      </c>
-      <c r="B97" t="b">
-        <v>1</v>
-      </c>
-      <c r="C97" t="n">
-        <v>1733</v>
-      </c>
-      <c r="D97" t="n">
-        <v>95.01000000000001</v>
-      </c>
-      <c r="E97" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>alter_fan</t>
-        </is>
-      </c>
-      <c r="B98" t="b">
-        <v>0</v>
-      </c>
-      <c r="C98" t="n">
-        <v>1730</v>
-      </c>
-      <c r="D98" t="n">
-        <v>94.84999999999999</v>
-      </c>
-      <c r="E98" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>_60950_1_2ed_A2</t>
-        </is>
-      </c>
-      <c r="B99" t="b">
-        <v>0</v>
-      </c>
-      <c r="C99" t="n">
-        <v>1717</v>
-      </c>
-      <c r="D99" t="n">
-        <v>94.13</v>
-      </c>
-      <c r="E99" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>11 (Ask Derek if  IEC/EN 62368-3  covers this)</t>
-        </is>
-      </c>
-      <c r="B100" t="b">
-        <v>0</v>
-      </c>
-      <c r="C100" t="n">
-        <v>1717</v>
-      </c>
-      <c r="D100" t="n">
-        <v>94.13</v>
-      </c>
-      <c r="E100" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>stalled_fan_test</t>
-        </is>
-      </c>
-      <c r="B101" t="b">
-        <v>0</v>
-      </c>
-      <c r="C101" t="n">
-        <v>1716</v>
-      </c>
-      <c r="D101" t="n">
-        <v>94.08</v>
-      </c>
-      <c r="E101" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>CCN_Top10_QQJQ</t>
-        </is>
-      </c>
-      <c r="B102" t="n">
-        <v>0</v>
-      </c>
-      <c r="C102" t="n">
-        <v>1701</v>
-      </c>
-      <c r="D102" t="n">
-        <v>93.26000000000001</v>
-      </c>
-      <c r="E102" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>CCN_Top10_QQJQ2</t>
-        </is>
-      </c>
-      <c r="B103" t="n">
-        <v>0</v>
-      </c>
-      <c r="C103" t="n">
-        <v>1700</v>
-      </c>
-      <c r="D103" t="n">
-        <v>93.2</v>
-      </c>
-      <c r="E103" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>blocked_vent_test</t>
-        </is>
-      </c>
-      <c r="B104" t="b">
-        <v>0</v>
-      </c>
-      <c r="C104" t="n">
-        <v>1698</v>
-      </c>
-      <c r="D104" t="n">
-        <v>93.09</v>
-      </c>
-      <c r="E104" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>1 (60950-1)</t>
-        </is>
-      </c>
-      <c r="B105" t="n">
-        <v>0</v>
-      </c>
-      <c r="C105" t="n">
-        <v>1695</v>
-      </c>
-      <c r="D105" t="n">
-        <v>92.93000000000001</v>
-      </c>
-      <c r="E105" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>CCN_Top10_AZOT2</t>
-        </is>
-      </c>
-      <c r="B106" t="n">
-        <v>0</v>
-      </c>
-      <c r="C106" t="n">
-        <v>1689</v>
-      </c>
-      <c r="D106" t="n">
-        <v>92.59999999999999</v>
-      </c>
-      <c r="E106" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>steady_force_test</t>
-        </is>
-      </c>
-      <c r="B107" t="b">
-        <v>0</v>
-      </c>
-      <c r="C107" t="n">
-        <v>1674</v>
-      </c>
-      <c r="D107" t="n">
-        <v>91.78</v>
-      </c>
-      <c r="E107" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>29 (Talk to Derek)</t>
-        </is>
-      </c>
-      <c r="B108" t="b">
-        <v>0</v>
-      </c>
-      <c r="C108" t="n">
-        <v>1669</v>
-      </c>
-      <c r="D108" t="n">
-        <v>91.5</v>
-      </c>
-      <c r="E108" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>capacitance_discharge_test</t>
-        </is>
-      </c>
-      <c r="B109" t="b">
-        <v>0</v>
-      </c>
-      <c r="C109" t="n">
-        <v>1648</v>
-      </c>
-      <c r="D109" t="n">
-        <v>90.34999999999999</v>
-      </c>
-      <c r="E109" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>touch_current_single_test</t>
-        </is>
-      </c>
-      <c r="B110" t="b">
-        <v>0</v>
-      </c>
-      <c r="C110" t="n">
-        <v>1644</v>
-      </c>
-      <c r="D110" t="n">
-        <v>90.13</v>
-      </c>
-      <c r="E110" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>